<commit_message>
rev subject no reparables
</commit_message>
<xml_diff>
--- a/backend/templates/NotasCert_Template.xlsx
+++ b/backend/templates/NotasCert_Template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D80E0BB1-4C40-424E-864F-13B028E7CA64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C84E9365-F56D-4C4E-8B69-25026F8BC1BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -702,7 +702,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -732,18 +732,92 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" shrinkToFit="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -755,16 +829,7 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -772,71 +837,17 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" shrinkToFit="1"/>
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1256,352 +1267,352 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" s="2" customFormat="1" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J1" s="41" t="s">
+      <c r="J1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="K1" s="41"/>
-      <c r="L1" s="41"/>
-      <c r="M1" s="41"/>
-      <c r="N1" s="41"/>
-      <c r="O1" s="41"/>
-      <c r="P1" s="41"/>
-      <c r="Q1" s="41"/>
-      <c r="R1" s="41"/>
-      <c r="S1" s="41"/>
-      <c r="T1" s="41"/>
-      <c r="U1" s="41"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
+      <c r="O1" s="13"/>
+      <c r="P1" s="13"/>
+      <c r="Q1" s="13"/>
+      <c r="R1" s="13"/>
+      <c r="S1" s="13"/>
+      <c r="T1" s="13"/>
+      <c r="U1" s="13"/>
     </row>
     <row r="2" spans="1:21" s="2" customFormat="1" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="K2" s="42" t="s">
+      <c r="K2" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="L2" s="42"/>
-      <c r="M2" s="42"/>
-      <c r="N2" s="43" t="s">
+      <c r="L2" s="14"/>
+      <c r="M2" s="14"/>
+      <c r="N2" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="O2" s="43"/>
-      <c r="P2" s="43"/>
-      <c r="Q2" s="43"/>
-      <c r="R2" s="27" t="s">
+      <c r="O2" s="15"/>
+      <c r="P2" s="15"/>
+      <c r="Q2" s="15"/>
+      <c r="R2" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="S2" s="27"/>
-      <c r="T2" s="44"/>
-      <c r="U2" s="44"/>
+      <c r="S2" s="16"/>
+      <c r="T2" s="17"/>
+      <c r="U2" s="17"/>
     </row>
     <row r="3" spans="1:21" s="2" customFormat="1" ht="12.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J3" s="45" t="s">
+      <c r="J3" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="K3" s="45"/>
-      <c r="L3" s="45"/>
-      <c r="M3" s="45"/>
-      <c r="N3" s="46"/>
-      <c r="O3" s="46"/>
-      <c r="P3" s="46"/>
-      <c r="Q3" s="46"/>
-      <c r="R3" s="46"/>
-      <c r="S3" s="46"/>
-      <c r="T3" s="46"/>
-      <c r="U3" s="46"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
+      <c r="M3" s="18"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="19"/>
+      <c r="P3" s="19"/>
+      <c r="Q3" s="19"/>
+      <c r="R3" s="19"/>
+      <c r="S3" s="19"/>
+      <c r="T3" s="19"/>
+      <c r="U3" s="19"/>
     </row>
     <row r="4" spans="1:21" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A5" s="32" t="s">
+      <c r="A5" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="32"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="32"/>
-      <c r="G5" s="32"/>
-      <c r="H5" s="32"/>
-      <c r="I5" s="32"/>
-      <c r="J5" s="32"/>
-      <c r="K5" s="32"/>
-      <c r="L5" s="32"/>
-      <c r="M5" s="32"/>
-      <c r="N5" s="32"/>
-      <c r="O5" s="32"/>
-      <c r="P5" s="32"/>
-      <c r="Q5" s="32"/>
-      <c r="R5" s="32"/>
-      <c r="S5" s="32"/>
-      <c r="T5" s="32"/>
-      <c r="U5" s="32"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20"/>
+      <c r="H5" s="20"/>
+      <c r="I5" s="20"/>
+      <c r="J5" s="20"/>
+      <c r="K5" s="20"/>
+      <c r="L5" s="20"/>
+      <c r="M5" s="20"/>
+      <c r="N5" s="20"/>
+      <c r="O5" s="20"/>
+      <c r="P5" s="20"/>
+      <c r="Q5" s="20"/>
+      <c r="R5" s="20"/>
+      <c r="S5" s="20"/>
+      <c r="T5" s="20"/>
+      <c r="U5" s="20"/>
     </row>
     <row r="6" spans="1:21" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="35"/>
-      <c r="C6" s="35"/>
-      <c r="D6" s="37" t="s">
+      <c r="B6" s="21"/>
+      <c r="C6" s="21"/>
+      <c r="D6" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="37"/>
-      <c r="F6" s="37"/>
-      <c r="G6" s="37"/>
-      <c r="H6" s="37"/>
-      <c r="I6" s="35"/>
-      <c r="J6" s="35"/>
-      <c r="K6" s="35"/>
-      <c r="L6" s="35"/>
-      <c r="M6" s="35"/>
-      <c r="N6" s="35"/>
-      <c r="O6" s="35"/>
-      <c r="P6" s="35"/>
-      <c r="Q6" s="35"/>
-      <c r="R6" s="35"/>
-      <c r="S6" s="35"/>
-      <c r="T6" s="35"/>
-      <c r="U6" s="35"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="22"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="21"/>
+      <c r="K6" s="21"/>
+      <c r="L6" s="21"/>
+      <c r="M6" s="21"/>
+      <c r="N6" s="21"/>
+      <c r="O6" s="21"/>
+      <c r="P6" s="21"/>
+      <c r="Q6" s="21"/>
+      <c r="R6" s="21"/>
+      <c r="S6" s="21"/>
+      <c r="T6" s="21"/>
+      <c r="U6" s="21"/>
     </row>
     <row r="7" spans="1:21" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="35"/>
-      <c r="D7" s="35"/>
-      <c r="E7" s="35"/>
-      <c r="F7" s="35"/>
-      <c r="G7" s="35"/>
-      <c r="H7" s="35"/>
-      <c r="I7" s="35"/>
-      <c r="J7" s="35"/>
-      <c r="K7" s="35"/>
-      <c r="L7" s="35"/>
-      <c r="M7" s="35"/>
-      <c r="N7" s="35"/>
-      <c r="O7" s="39" t="s">
+      <c r="C7" s="21"/>
+      <c r="D7" s="21"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="21"/>
+      <c r="H7" s="21"/>
+      <c r="I7" s="21"/>
+      <c r="J7" s="21"/>
+      <c r="K7" s="21"/>
+      <c r="L7" s="21"/>
+      <c r="M7" s="21"/>
+      <c r="N7" s="21"/>
+      <c r="O7" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="P7" s="39"/>
-      <c r="Q7" s="36"/>
-      <c r="R7" s="36"/>
-      <c r="S7" s="36"/>
-      <c r="T7" s="36"/>
-      <c r="U7" s="36"/>
+      <c r="P7" s="23"/>
+      <c r="Q7" s="24"/>
+      <c r="R7" s="24"/>
+      <c r="S7" s="24"/>
+      <c r="T7" s="24"/>
+      <c r="U7" s="24"/>
     </row>
     <row r="8" spans="1:21" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="36"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="36"/>
-      <c r="F8" s="36"/>
-      <c r="G8" s="36"/>
-      <c r="H8" s="36"/>
-      <c r="M8" s="36"/>
-      <c r="N8" s="36"/>
-      <c r="O8" s="39" t="s">
+      <c r="C8" s="24"/>
+      <c r="D8" s="24"/>
+      <c r="E8" s="24"/>
+      <c r="F8" s="24"/>
+      <c r="G8" s="24"/>
+      <c r="H8" s="24"/>
+      <c r="M8" s="24"/>
+      <c r="N8" s="24"/>
+      <c r="O8" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="P8" s="39"/>
-      <c r="Q8" s="35"/>
-      <c r="R8" s="35"/>
-      <c r="S8" s="35"/>
-      <c r="T8" s="35"/>
-      <c r="U8" s="35"/>
+      <c r="P8" s="23"/>
+      <c r="Q8" s="21"/>
+      <c r="R8" s="21"/>
+      <c r="S8" s="21"/>
+      <c r="T8" s="21"/>
+      <c r="U8" s="21"/>
     </row>
     <row r="9" spans="1:21" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="32" t="s">
+      <c r="A9" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="32"/>
-      <c r="C9" s="32"/>
-      <c r="D9" s="32"/>
-      <c r="E9" s="32"/>
-      <c r="F9" s="32"/>
-      <c r="G9" s="32"/>
-      <c r="H9" s="32"/>
-      <c r="I9" s="32"/>
-      <c r="J9" s="32"/>
-      <c r="K9" s="32"/>
-      <c r="L9" s="32"/>
-      <c r="M9" s="32"/>
-      <c r="N9" s="32"/>
-      <c r="O9" s="32"/>
-      <c r="P9" s="32"/>
-      <c r="Q9" s="32"/>
-      <c r="R9" s="32"/>
-      <c r="S9" s="32"/>
-      <c r="T9" s="32"/>
-      <c r="U9" s="32"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="20"/>
+      <c r="J9" s="20"/>
+      <c r="K9" s="20"/>
+      <c r="L9" s="20"/>
+      <c r="M9" s="20"/>
+      <c r="N9" s="20"/>
+      <c r="O9" s="20"/>
+      <c r="P9" s="20"/>
+      <c r="Q9" s="20"/>
+      <c r="R9" s="20"/>
+      <c r="S9" s="20"/>
+      <c r="T9" s="20"/>
+      <c r="U9" s="20"/>
     </row>
     <row r="10" spans="1:21" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="40" t="s">
+      <c r="A10" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="40"/>
-      <c r="C10" s="35"/>
-      <c r="D10" s="35"/>
-      <c r="E10" s="35"/>
+      <c r="B10" s="25"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="21"/>
       <c r="F10" s="6"/>
-      <c r="H10" s="37" t="s">
+      <c r="H10" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="I10" s="37"/>
-      <c r="J10" s="37"/>
-      <c r="K10" s="37"/>
-      <c r="L10" s="37"/>
-      <c r="M10" s="35"/>
-      <c r="N10" s="35"/>
-      <c r="O10" s="35"/>
-      <c r="P10" s="35"/>
-      <c r="Q10" s="35"/>
-      <c r="R10" s="35"/>
-      <c r="S10" s="35"/>
-      <c r="T10" s="35"/>
-      <c r="U10" s="35"/>
+      <c r="I10" s="22"/>
+      <c r="J10" s="22"/>
+      <c r="K10" s="22"/>
+      <c r="L10" s="22"/>
+      <c r="M10" s="21"/>
+      <c r="N10" s="21"/>
+      <c r="O10" s="21"/>
+      <c r="P10" s="21"/>
+      <c r="Q10" s="21"/>
+      <c r="R10" s="21"/>
+      <c r="S10" s="21"/>
+      <c r="T10" s="21"/>
+      <c r="U10" s="21"/>
     </row>
     <row r="11" spans="1:21" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="35"/>
-      <c r="C11" s="35"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="35"/>
-      <c r="F11" s="35"/>
-      <c r="G11" s="35"/>
-      <c r="H11" s="35"/>
-      <c r="I11" s="35"/>
-      <c r="J11" s="35"/>
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
+      <c r="D11" s="21"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="21"/>
+      <c r="H11" s="21"/>
+      <c r="I11" s="21"/>
+      <c r="J11" s="21"/>
       <c r="L11" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="M11" s="36"/>
-      <c r="N11" s="36"/>
-      <c r="O11" s="36"/>
-      <c r="P11" s="36"/>
-      <c r="Q11" s="36"/>
-      <c r="R11" s="36"/>
-      <c r="S11" s="36"/>
-      <c r="T11" s="36"/>
-      <c r="U11" s="36"/>
-    </row>
-    <row r="12" spans="1:21" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M11" s="24"/>
+      <c r="N11" s="24"/>
+      <c r="O11" s="24"/>
+      <c r="P11" s="24"/>
+      <c r="Q11" s="24"/>
+      <c r="R11" s="24"/>
+      <c r="S11" s="24"/>
+      <c r="T11" s="24"/>
+      <c r="U11" s="24"/>
+    </row>
+    <row r="12" spans="1:21" ht="12.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="36"/>
-      <c r="E12" s="36"/>
-      <c r="F12" s="36"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="24"/>
       <c r="G12" s="6"/>
-      <c r="H12" s="37" t="s">
+      <c r="H12" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="I12" s="37"/>
-      <c r="J12" s="35"/>
-      <c r="K12" s="35"/>
-      <c r="L12" s="32"/>
-      <c r="M12" s="32"/>
+      <c r="I12" s="22"/>
+      <c r="J12" s="21"/>
+      <c r="K12" s="21"/>
+      <c r="L12" s="20"/>
+      <c r="M12" s="20"/>
       <c r="N12" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="O12" s="32"/>
-      <c r="P12" s="32"/>
-      <c r="Q12" s="32"/>
-      <c r="R12" s="32"/>
-      <c r="S12" s="32"/>
-      <c r="T12" s="32"/>
-      <c r="U12" s="32"/>
-    </row>
-    <row r="13" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="38" t="s">
+      <c r="O12" s="20"/>
+      <c r="P12" s="20"/>
+      <c r="Q12" s="20"/>
+      <c r="R12" s="20"/>
+      <c r="S12" s="20"/>
+      <c r="T12" s="20"/>
+      <c r="U12" s="20"/>
+    </row>
+    <row r="13" spans="1:21" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="38"/>
-      <c r="C13" s="38"/>
-      <c r="D13" s="38"/>
-      <c r="E13" s="38"/>
-      <c r="F13" s="38"/>
-      <c r="G13" s="38"/>
-      <c r="H13" s="38"/>
-      <c r="I13" s="38"/>
-      <c r="J13" s="38"/>
+      <c r="B13" s="26"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="26"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="26"/>
+      <c r="J13" s="26"/>
       <c r="K13" s="7"/>
       <c r="L13" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="M13" s="33" t="s">
+      <c r="M13" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="N13" s="33"/>
-      <c r="O13" s="33"/>
-      <c r="P13" s="33"/>
-      <c r="Q13" s="33" t="s">
+      <c r="N13" s="27"/>
+      <c r="O13" s="27"/>
+      <c r="P13" s="27"/>
+      <c r="Q13" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="R13" s="33"/>
-      <c r="S13" s="33"/>
-      <c r="T13" s="33"/>
-      <c r="U13" s="8" t="s">
+      <c r="R13" s="27"/>
+      <c r="S13" s="27"/>
+      <c r="T13" s="27"/>
+      <c r="U13" s="46" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="33" t="s">
+      <c r="B14" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="33"/>
-      <c r="D14" s="33"/>
-      <c r="E14" s="33"/>
-      <c r="F14" s="33"/>
-      <c r="G14" s="33" t="s">
+      <c r="C14" s="27"/>
+      <c r="D14" s="27"/>
+      <c r="E14" s="27"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="H14" s="33"/>
-      <c r="I14" s="33"/>
-      <c r="J14" s="8" t="s">
+      <c r="H14" s="27"/>
+      <c r="I14" s="27"/>
+      <c r="J14" s="46" t="s">
         <v>23</v>
       </c>
       <c r="K14" s="7"/>
       <c r="L14" s="8">
         <v>3</v>
       </c>
-      <c r="M14" s="34" t="s">
+      <c r="M14" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="N14" s="34"/>
-      <c r="O14" s="34"/>
-      <c r="P14" s="34"/>
-      <c r="Q14" s="34" t="s">
+      <c r="N14" s="28"/>
+      <c r="O14" s="28"/>
+      <c r="P14" s="28"/>
+      <c r="Q14" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="R14" s="34"/>
-      <c r="S14" s="34"/>
-      <c r="T14" s="34"/>
+      <c r="R14" s="28"/>
+      <c r="S14" s="28"/>
+      <c r="T14" s="28"/>
       <c r="U14" s="8" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="15" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="34" t="s">
+      <c r="B15" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="C15" s="34"/>
-      <c r="D15" s="34"/>
-      <c r="E15" s="34"/>
-      <c r="F15" s="34"/>
-      <c r="G15" s="34" t="s">
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="28"/>
+      <c r="G15" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="H15" s="34"/>
-      <c r="I15" s="34"/>
+      <c r="H15" s="28"/>
+      <c r="I15" s="28"/>
       <c r="J15" s="8" t="s">
         <v>62</v>
       </c>
@@ -1609,18 +1620,18 @@
       <c r="L15" s="8">
         <v>4</v>
       </c>
-      <c r="M15" s="34" t="s">
+      <c r="M15" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="N15" s="34"/>
-      <c r="O15" s="34"/>
-      <c r="P15" s="34"/>
-      <c r="Q15" s="34" t="s">
+      <c r="N15" s="28"/>
+      <c r="O15" s="28"/>
+      <c r="P15" s="28"/>
+      <c r="Q15" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="R15" s="34"/>
-      <c r="S15" s="34"/>
-      <c r="T15" s="34"/>
+      <c r="R15" s="28"/>
+      <c r="S15" s="28"/>
+      <c r="T15" s="28"/>
       <c r="U15" s="8" t="s">
         <v>62</v>
       </c>
@@ -1629,18 +1640,18 @@
       <c r="A16" s="8">
         <v>2</v>
       </c>
-      <c r="B16" s="34" t="s">
+      <c r="B16" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="C16" s="34"/>
-      <c r="D16" s="34"/>
-      <c r="E16" s="34"/>
-      <c r="F16" s="34"/>
-      <c r="G16" s="34" t="s">
+      <c r="C16" s="28"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="28"/>
+      <c r="G16" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="H16" s="34"/>
-      <c r="I16" s="34"/>
+      <c r="H16" s="28"/>
+      <c r="I16" s="28"/>
       <c r="J16" s="8" t="s">
         <v>62</v>
       </c>
@@ -1648,167 +1659,167 @@
       <c r="L16" s="8">
         <v>5</v>
       </c>
-      <c r="M16" s="34" t="s">
+      <c r="M16" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="N16" s="34"/>
-      <c r="O16" s="34"/>
-      <c r="P16" s="34"/>
-      <c r="Q16" s="34" t="s">
+      <c r="N16" s="28"/>
+      <c r="O16" s="28"/>
+      <c r="P16" s="28"/>
+      <c r="Q16" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="R16" s="34"/>
-      <c r="S16" s="34"/>
-      <c r="T16" s="34"/>
+      <c r="R16" s="28"/>
+      <c r="S16" s="28"/>
+      <c r="T16" s="28"/>
       <c r="U16" s="8" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A17" s="32" t="s">
+      <c r="A17" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="32"/>
-      <c r="C17" s="32"/>
-      <c r="D17" s="32"/>
-      <c r="E17" s="32"/>
-      <c r="F17" s="32"/>
-      <c r="G17" s="32"/>
-      <c r="H17" s="32"/>
-      <c r="I17" s="32"/>
-      <c r="J17" s="32"/>
-      <c r="K17" s="32"/>
-      <c r="L17" s="32"/>
-      <c r="M17" s="32"/>
-      <c r="N17" s="32"/>
-      <c r="O17" s="32"/>
-      <c r="P17" s="32"/>
-      <c r="Q17" s="32"/>
-      <c r="R17" s="32"/>
-      <c r="S17" s="32"/>
-      <c r="T17" s="32"/>
-      <c r="U17" s="32"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="20"/>
+      <c r="G17" s="20"/>
+      <c r="H17" s="20"/>
+      <c r="I17" s="20"/>
+      <c r="J17" s="20"/>
+      <c r="K17" s="20"/>
+      <c r="L17" s="20"/>
+      <c r="M17" s="20"/>
+      <c r="N17" s="20"/>
+      <c r="O17" s="20"/>
+      <c r="P17" s="20"/>
+      <c r="Q17" s="20"/>
+      <c r="R17" s="20"/>
+      <c r="S17" s="20"/>
+      <c r="T17" s="20"/>
+      <c r="U17" s="20"/>
     </row>
     <row r="18" spans="1:21" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="27" t="s">
+      <c r="A18" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="27"/>
-      <c r="C18" s="27"/>
-      <c r="D18" s="27"/>
-      <c r="E18" s="27"/>
-      <c r="F18" s="27"/>
-      <c r="G18" s="27"/>
-      <c r="H18" s="27"/>
-      <c r="I18" s="27"/>
-      <c r="J18" s="27"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="16"/>
       <c r="K18" s="3"/>
-      <c r="L18" s="27" t="s">
+      <c r="L18" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="M18" s="27"/>
-      <c r="N18" s="27"/>
-      <c r="O18" s="27"/>
-      <c r="P18" s="27"/>
-      <c r="Q18" s="27"/>
-      <c r="R18" s="27"/>
-      <c r="S18" s="27"/>
-      <c r="T18" s="27"/>
-      <c r="U18" s="27"/>
+      <c r="M18" s="16"/>
+      <c r="N18" s="16"/>
+      <c r="O18" s="16"/>
+      <c r="P18" s="16"/>
+      <c r="Q18" s="16"/>
+      <c r="R18" s="16"/>
+      <c r="S18" s="16"/>
+      <c r="T18" s="16"/>
+      <c r="U18" s="16"/>
     </row>
     <row r="19" spans="1:21" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="19" t="s">
+      <c r="A19" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="B19" s="19"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="26" t="s">
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="19" t="s">
+      <c r="E19" s="30"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="H19" s="26" t="s">
+      <c r="H19" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="I19" s="26"/>
-      <c r="J19" s="28" t="s">
+      <c r="I19" s="30"/>
+      <c r="J19" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="L19" s="19" t="s">
+      <c r="L19" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="M19" s="19"/>
-      <c r="N19" s="19"/>
-      <c r="O19" s="26" t="s">
+      <c r="M19" s="29"/>
+      <c r="N19" s="29"/>
+      <c r="O19" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="P19" s="26"/>
-      <c r="Q19" s="19" t="s">
+      <c r="P19" s="30"/>
+      <c r="Q19" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="R19" s="26" t="s">
+      <c r="R19" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="S19" s="26"/>
-      <c r="T19" s="26"/>
-      <c r="U19" s="28" t="s">
+      <c r="S19" s="30"/>
+      <c r="T19" s="30"/>
+      <c r="U19" s="31" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="20" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="19"/>
-      <c r="B20" s="19"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="9" t="s">
+      <c r="A20" s="29"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="E20" s="19" t="s">
+      <c r="E20" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="F20" s="19"/>
-      <c r="G20" s="19"/>
-      <c r="H20" s="9" t="s">
+      <c r="F20" s="29"/>
+      <c r="G20" s="47"/>
+      <c r="H20" s="46" t="s">
         <v>33</v>
       </c>
-      <c r="I20" s="9" t="s">
+      <c r="I20" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="J20" s="28"/>
-      <c r="L20" s="19"/>
-      <c r="M20" s="19"/>
-      <c r="N20" s="19"/>
-      <c r="O20" s="9" t="s">
+      <c r="J20" s="31"/>
+      <c r="L20" s="29"/>
+      <c r="M20" s="29"/>
+      <c r="N20" s="29"/>
+      <c r="O20" s="46" t="s">
         <v>20</v>
       </c>
       <c r="P20" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="Q20" s="19"/>
-      <c r="R20" s="9" t="s">
+      <c r="Q20" s="47"/>
+      <c r="R20" s="46" t="s">
         <v>33</v>
       </c>
-      <c r="S20" s="19" t="s">
+      <c r="S20" s="47" t="s">
         <v>34</v>
       </c>
-      <c r="T20" s="19"/>
-      <c r="U20" s="28"/>
+      <c r="T20" s="47"/>
+      <c r="U20" s="31"/>
     </row>
     <row r="21" spans="1:21" ht="12" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="B21" s="15"/>
-      <c r="C21" s="15"/>
+      <c r="A21" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="B21" s="32"/>
+      <c r="C21" s="32"/>
       <c r="D21" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E21" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F21" s="25"/>
+      <c r="E21" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F21" s="33"/>
       <c r="G21" s="10" t="s">
         <v>65</v>
       </c>
@@ -1821,15 +1832,15 @@
       <c r="J21" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L21" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="M21" s="25"/>
-      <c r="N21" s="25"/>
+      <c r="L21" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="M21" s="33"/>
+      <c r="N21" s="33"/>
       <c r="O21" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="P21" s="13" t="s">
+      <c r="P21" s="12" t="s">
         <v>66</v>
       </c>
       <c r="Q21" s="10" t="s">
@@ -1838,27 +1849,27 @@
       <c r="R21" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="S21" s="30" t="s">
-        <v>63</v>
-      </c>
-      <c r="T21" s="31"/>
+      <c r="S21" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="T21" s="35"/>
       <c r="U21" s="10" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="22" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="B22" s="15"/>
-      <c r="C22" s="15"/>
+      <c r="A22" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="B22" s="32"/>
+      <c r="C22" s="32"/>
       <c r="D22" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E22" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F22" s="25"/>
+      <c r="E22" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F22" s="33"/>
       <c r="G22" s="10" t="s">
         <v>65</v>
       </c>
@@ -1871,15 +1882,15 @@
       <c r="J22" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L22" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="M22" s="25"/>
-      <c r="N22" s="25"/>
+      <c r="L22" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="M22" s="33"/>
+      <c r="N22" s="33"/>
       <c r="O22" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="P22" s="13" t="s">
+      <c r="P22" s="12" t="s">
         <v>66</v>
       </c>
       <c r="Q22" s="10" t="s">
@@ -1888,27 +1899,27 @@
       <c r="R22" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="S22" s="30" t="s">
-        <v>63</v>
-      </c>
-      <c r="T22" s="31"/>
+      <c r="S22" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="T22" s="35"/>
       <c r="U22" s="10" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="23" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="B23" s="15"/>
-      <c r="C23" s="15"/>
+      <c r="A23" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="B23" s="32"/>
+      <c r="C23" s="32"/>
       <c r="D23" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E23" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F23" s="25"/>
+      <c r="E23" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F23" s="33"/>
       <c r="G23" s="10" t="s">
         <v>65</v>
       </c>
@@ -1921,15 +1932,15 @@
       <c r="J23" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L23" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="M23" s="25"/>
-      <c r="N23" s="25"/>
+      <c r="L23" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="M23" s="33"/>
+      <c r="N23" s="33"/>
       <c r="O23" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="P23" s="13" t="s">
+      <c r="P23" s="12" t="s">
         <v>66</v>
       </c>
       <c r="Q23" s="10" t="s">
@@ -1938,27 +1949,27 @@
       <c r="R23" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="S23" s="30" t="s">
-        <v>63</v>
-      </c>
-      <c r="T23" s="31"/>
+      <c r="S23" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="T23" s="35"/>
       <c r="U23" s="10" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="24" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="B24" s="15"/>
-      <c r="C24" s="15"/>
+      <c r="A24" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="B24" s="32"/>
+      <c r="C24" s="32"/>
       <c r="D24" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E24" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F24" s="25"/>
+      <c r="E24" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F24" s="33"/>
       <c r="G24" s="10" t="s">
         <v>65</v>
       </c>
@@ -1971,15 +1982,15 @@
       <c r="J24" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L24" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="M24" s="25"/>
-      <c r="N24" s="25"/>
+      <c r="L24" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="M24" s="33"/>
+      <c r="N24" s="33"/>
       <c r="O24" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="P24" s="13" t="s">
+      <c r="P24" s="12" t="s">
         <v>66</v>
       </c>
       <c r="Q24" s="10" t="s">
@@ -1988,27 +1999,27 @@
       <c r="R24" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="S24" s="30" t="s">
-        <v>63</v>
-      </c>
-      <c r="T24" s="31"/>
+      <c r="S24" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="T24" s="35"/>
       <c r="U24" s="10" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="25" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="B25" s="15"/>
-      <c r="C25" s="15"/>
+      <c r="A25" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="B25" s="32"/>
+      <c r="C25" s="32"/>
       <c r="D25" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E25" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F25" s="25"/>
+      <c r="E25" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F25" s="33"/>
       <c r="G25" s="10" t="s">
         <v>65</v>
       </c>
@@ -2021,15 +2032,15 @@
       <c r="J25" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L25" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="M25" s="25"/>
-      <c r="N25" s="25"/>
+      <c r="L25" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="M25" s="33"/>
+      <c r="N25" s="33"/>
       <c r="O25" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="P25" s="13" t="s">
+      <c r="P25" s="12" t="s">
         <v>66</v>
       </c>
       <c r="Q25" s="10" t="s">
@@ -2038,27 +2049,27 @@
       <c r="R25" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="S25" s="30" t="s">
-        <v>63</v>
-      </c>
-      <c r="T25" s="31"/>
+      <c r="S25" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="T25" s="35"/>
       <c r="U25" s="10" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="26" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="B26" s="15"/>
-      <c r="C26" s="15"/>
+      <c r="A26" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="B26" s="32"/>
+      <c r="C26" s="32"/>
       <c r="D26" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E26" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F26" s="25"/>
+      <c r="E26" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F26" s="33"/>
       <c r="G26" s="10" t="s">
         <v>65</v>
       </c>
@@ -2071,15 +2082,15 @@
       <c r="J26" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L26" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="M26" s="25"/>
-      <c r="N26" s="25"/>
+      <c r="L26" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="M26" s="33"/>
+      <c r="N26" s="33"/>
       <c r="O26" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="P26" s="13" t="s">
+      <c r="P26" s="12" t="s">
         <v>66</v>
       </c>
       <c r="Q26" s="10" t="s">
@@ -2088,27 +2099,27 @@
       <c r="R26" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="S26" s="30" t="s">
-        <v>63</v>
-      </c>
-      <c r="T26" s="31"/>
+      <c r="S26" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="T26" s="35"/>
       <c r="U26" s="10" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="27" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="B27" s="15"/>
-      <c r="C27" s="15"/>
+      <c r="A27" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="B27" s="32"/>
+      <c r="C27" s="32"/>
       <c r="D27" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E27" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F27" s="25"/>
+      <c r="E27" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F27" s="33"/>
       <c r="G27" s="10" t="s">
         <v>65</v>
       </c>
@@ -2121,15 +2132,15 @@
       <c r="J27" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L27" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="M27" s="25"/>
-      <c r="N27" s="25"/>
+      <c r="L27" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="M27" s="33"/>
+      <c r="N27" s="33"/>
       <c r="O27" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="P27" s="13" t="s">
+      <c r="P27" s="12" t="s">
         <v>66</v>
       </c>
       <c r="Q27" s="10" t="s">
@@ -2138,134 +2149,134 @@
       <c r="R27" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="S27" s="30" t="s">
-        <v>63</v>
-      </c>
-      <c r="T27" s="31"/>
+      <c r="S27" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="T27" s="35"/>
       <c r="U27" s="10" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="28" spans="1:21" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="27" t="s">
+      <c r="A28" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="B28" s="27"/>
-      <c r="C28" s="27"/>
-      <c r="D28" s="27"/>
-      <c r="E28" s="27"/>
-      <c r="F28" s="27"/>
-      <c r="G28" s="27"/>
-      <c r="H28" s="27"/>
-      <c r="I28" s="27"/>
-      <c r="J28" s="27"/>
+      <c r="B28" s="16"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="16"/>
+      <c r="G28" s="16"/>
+      <c r="H28" s="16"/>
+      <c r="I28" s="16"/>
+      <c r="J28" s="16"/>
       <c r="K28" s="2"/>
-      <c r="L28" s="27" t="s">
+      <c r="L28" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="M28" s="27"/>
-      <c r="N28" s="27"/>
-      <c r="O28" s="27"/>
-      <c r="P28" s="27"/>
-      <c r="Q28" s="27"/>
-      <c r="R28" s="27"/>
-      <c r="S28" s="27"/>
-      <c r="T28" s="27"/>
-      <c r="U28" s="27"/>
+      <c r="M28" s="16"/>
+      <c r="N28" s="16"/>
+      <c r="O28" s="16"/>
+      <c r="P28" s="16"/>
+      <c r="Q28" s="16"/>
+      <c r="R28" s="16"/>
+      <c r="S28" s="16"/>
+      <c r="T28" s="16"/>
+      <c r="U28" s="16"/>
     </row>
     <row r="29" spans="1:21" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="19" t="s">
+      <c r="A29" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="19"/>
-      <c r="C29" s="19"/>
-      <c r="D29" s="26" t="s">
+      <c r="B29" s="29"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="E29" s="26"/>
-      <c r="F29" s="26"/>
-      <c r="G29" s="19" t="s">
+      <c r="E29" s="30"/>
+      <c r="F29" s="30"/>
+      <c r="G29" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="H29" s="26" t="s">
+      <c r="H29" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="I29" s="26"/>
-      <c r="J29" s="28" t="s">
+      <c r="I29" s="30"/>
+      <c r="J29" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="L29" s="19" t="s">
+      <c r="L29" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="M29" s="19"/>
-      <c r="N29" s="19"/>
-      <c r="O29" s="26" t="s">
+      <c r="M29" s="29"/>
+      <c r="N29" s="29"/>
+      <c r="O29" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="P29" s="26"/>
-      <c r="Q29" s="19" t="s">
+      <c r="P29" s="30"/>
+      <c r="Q29" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="R29" s="26" t="s">
+      <c r="R29" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="S29" s="26"/>
-      <c r="T29" s="26"/>
-      <c r="U29" s="28" t="s">
+      <c r="S29" s="30"/>
+      <c r="T29" s="30"/>
+      <c r="U29" s="31" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="30" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="19"/>
-      <c r="B30" s="19"/>
-      <c r="C30" s="19"/>
-      <c r="D30" s="9" t="s">
+      <c r="A30" s="29"/>
+      <c r="B30" s="29"/>
+      <c r="C30" s="29"/>
+      <c r="D30" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="E30" s="19" t="s">
+      <c r="E30" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="F30" s="19"/>
-      <c r="G30" s="19"/>
-      <c r="H30" s="9" t="s">
+      <c r="F30" s="29"/>
+      <c r="G30" s="47"/>
+      <c r="H30" s="46" t="s">
         <v>33</v>
       </c>
-      <c r="I30" s="9" t="s">
+      <c r="I30" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="J30" s="28"/>
-      <c r="L30" s="19"/>
-      <c r="M30" s="19"/>
-      <c r="N30" s="19"/>
-      <c r="O30" s="9" t="s">
+      <c r="J30" s="31"/>
+      <c r="L30" s="29"/>
+      <c r="M30" s="29"/>
+      <c r="N30" s="29"/>
+      <c r="O30" s="46" t="s">
         <v>20</v>
       </c>
       <c r="P30" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="Q30" s="19"/>
-      <c r="R30" s="9" t="s">
+      <c r="Q30" s="47"/>
+      <c r="R30" s="46" t="s">
         <v>33</v>
       </c>
-      <c r="S30" s="19" t="s">
+      <c r="S30" s="47" t="s">
         <v>34</v>
       </c>
-      <c r="T30" s="19"/>
-      <c r="U30" s="28"/>
+      <c r="T30" s="47"/>
+      <c r="U30" s="31"/>
     </row>
     <row r="31" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B31" s="25"/>
-      <c r="C31" s="25"/>
+      <c r="A31" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B31" s="33"/>
+      <c r="C31" s="33"/>
       <c r="D31" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E31" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F31" s="25"/>
+      <c r="E31" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F31" s="33"/>
       <c r="G31" s="10" t="s">
         <v>65</v>
       </c>
@@ -2278,15 +2289,15 @@
       <c r="J31" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L31" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="M31" s="25"/>
-      <c r="N31" s="25"/>
+      <c r="L31" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="M31" s="33"/>
+      <c r="N31" s="33"/>
       <c r="O31" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="P31" s="13" t="s">
+      <c r="P31" s="12" t="s">
         <v>66</v>
       </c>
       <c r="Q31" s="10" t="s">
@@ -2295,27 +2306,27 @@
       <c r="R31" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="S31" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="T31" s="14"/>
+      <c r="S31" s="36" t="s">
+        <v>63</v>
+      </c>
+      <c r="T31" s="36"/>
       <c r="U31" s="10" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="32" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B32" s="25"/>
-      <c r="C32" s="25"/>
+      <c r="A32" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B32" s="33"/>
+      <c r="C32" s="33"/>
       <c r="D32" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E32" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F32" s="25"/>
+      <c r="E32" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F32" s="33"/>
       <c r="G32" s="10" t="s">
         <v>65</v>
       </c>
@@ -2328,15 +2339,15 @@
       <c r="J32" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L32" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="M32" s="25"/>
-      <c r="N32" s="25"/>
+      <c r="L32" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="M32" s="33"/>
+      <c r="N32" s="33"/>
       <c r="O32" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="P32" s="13" t="s">
+      <c r="P32" s="12" t="s">
         <v>66</v>
       </c>
       <c r="Q32" s="10" t="s">
@@ -2345,27 +2356,27 @@
       <c r="R32" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="S32" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="T32" s="14"/>
+      <c r="S32" s="36" t="s">
+        <v>63</v>
+      </c>
+      <c r="T32" s="36"/>
       <c r="U32" s="10" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="33" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B33" s="25"/>
-      <c r="C33" s="25"/>
+      <c r="A33" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B33" s="33"/>
+      <c r="C33" s="33"/>
       <c r="D33" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E33" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F33" s="25"/>
+      <c r="E33" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F33" s="33"/>
       <c r="G33" s="10" t="s">
         <v>65</v>
       </c>
@@ -2378,15 +2389,15 @@
       <c r="J33" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L33" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="M33" s="25"/>
-      <c r="N33" s="25"/>
+      <c r="L33" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="M33" s="33"/>
+      <c r="N33" s="33"/>
       <c r="O33" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="P33" s="13" t="s">
+      <c r="P33" s="12" t="s">
         <v>66</v>
       </c>
       <c r="Q33" s="10" t="s">
@@ -2395,27 +2406,27 @@
       <c r="R33" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="S33" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="T33" s="14"/>
+      <c r="S33" s="36" t="s">
+        <v>63</v>
+      </c>
+      <c r="T33" s="36"/>
       <c r="U33" s="10" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="34" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B34" s="25"/>
-      <c r="C34" s="25"/>
+      <c r="A34" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B34" s="33"/>
+      <c r="C34" s="33"/>
       <c r="D34" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E34" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F34" s="25"/>
+      <c r="E34" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F34" s="33"/>
       <c r="G34" s="10" t="s">
         <v>65</v>
       </c>
@@ -2428,15 +2439,15 @@
       <c r="J34" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L34" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="M34" s="25"/>
-      <c r="N34" s="25"/>
+      <c r="L34" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="M34" s="33"/>
+      <c r="N34" s="33"/>
       <c r="O34" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="P34" s="13" t="s">
+      <c r="P34" s="12" t="s">
         <v>66</v>
       </c>
       <c r="Q34" s="10" t="s">
@@ -2445,27 +2456,27 @@
       <c r="R34" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="S34" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="T34" s="14"/>
+      <c r="S34" s="36" t="s">
+        <v>63</v>
+      </c>
+      <c r="T34" s="36"/>
       <c r="U34" s="10" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="35" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B35" s="25"/>
-      <c r="C35" s="25"/>
+      <c r="A35" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B35" s="33"/>
+      <c r="C35" s="33"/>
       <c r="D35" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E35" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F35" s="25"/>
+      <c r="E35" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F35" s="33"/>
       <c r="G35" s="10" t="s">
         <v>65</v>
       </c>
@@ -2478,15 +2489,15 @@
       <c r="J35" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L35" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="M35" s="25"/>
-      <c r="N35" s="25"/>
+      <c r="L35" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="M35" s="33"/>
+      <c r="N35" s="33"/>
       <c r="O35" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="P35" s="13" t="s">
+      <c r="P35" s="12" t="s">
         <v>66</v>
       </c>
       <c r="Q35" s="10" t="s">
@@ -2495,27 +2506,27 @@
       <c r="R35" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="S35" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="T35" s="14"/>
+      <c r="S35" s="36" t="s">
+        <v>63</v>
+      </c>
+      <c r="T35" s="36"/>
       <c r="U35" s="10" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="36" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B36" s="25"/>
-      <c r="C36" s="25"/>
+      <c r="A36" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B36" s="33"/>
+      <c r="C36" s="33"/>
       <c r="D36" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E36" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F36" s="25"/>
+      <c r="E36" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F36" s="33"/>
       <c r="G36" s="10" t="s">
         <v>65</v>
       </c>
@@ -2528,15 +2539,15 @@
       <c r="J36" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L36" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="M36" s="25"/>
-      <c r="N36" s="25"/>
+      <c r="L36" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="M36" s="33"/>
+      <c r="N36" s="33"/>
       <c r="O36" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="P36" s="13" t="s">
+      <c r="P36" s="12" t="s">
         <v>66</v>
       </c>
       <c r="Q36" s="10" t="s">
@@ -2545,27 +2556,27 @@
       <c r="R36" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="S36" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="T36" s="14"/>
+      <c r="S36" s="36" t="s">
+        <v>63</v>
+      </c>
+      <c r="T36" s="36"/>
       <c r="U36" s="10" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="37" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B37" s="25"/>
-      <c r="C37" s="25"/>
+      <c r="A37" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B37" s="33"/>
+      <c r="C37" s="33"/>
       <c r="D37" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E37" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F37" s="25"/>
+      <c r="E37" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F37" s="33"/>
       <c r="G37" s="10" t="s">
         <v>65</v>
       </c>
@@ -2578,15 +2589,15 @@
       <c r="J37" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L37" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="M37" s="25"/>
-      <c r="N37" s="25"/>
+      <c r="L37" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="M37" s="33"/>
+      <c r="N37" s="33"/>
       <c r="O37" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="P37" s="13" t="s">
+      <c r="P37" s="12" t="s">
         <v>66</v>
       </c>
       <c r="Q37" s="10" t="s">
@@ -2595,27 +2606,27 @@
       <c r="R37" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="S37" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="T37" s="14"/>
+      <c r="S37" s="36" t="s">
+        <v>63</v>
+      </c>
+      <c r="T37" s="36"/>
       <c r="U37" s="10" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="38" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B38" s="25"/>
-      <c r="C38" s="25"/>
+      <c r="A38" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B38" s="33"/>
+      <c r="C38" s="33"/>
       <c r="D38" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E38" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F38" s="25"/>
+      <c r="E38" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F38" s="33"/>
       <c r="G38" s="10" t="s">
         <v>65</v>
       </c>
@@ -2628,15 +2639,15 @@
       <c r="J38" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L38" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="M38" s="25"/>
-      <c r="N38" s="25"/>
+      <c r="L38" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="M38" s="33"/>
+      <c r="N38" s="33"/>
       <c r="O38" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="P38" s="13" t="s">
+      <c r="P38" s="12" t="s">
         <v>66</v>
       </c>
       <c r="Q38" s="10" t="s">
@@ -2645,28 +2656,28 @@
       <c r="R38" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="S38" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="T38" s="14"/>
+      <c r="S38" s="36" t="s">
+        <v>63</v>
+      </c>
+      <c r="T38" s="36"/>
       <c r="U38" s="10" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="39" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="29"/>
-      <c r="B39" s="29"/>
-      <c r="E39" s="29"/>
-      <c r="F39" s="29"/>
-      <c r="L39" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="M39" s="25"/>
-      <c r="N39" s="25"/>
+      <c r="A39" s="37"/>
+      <c r="B39" s="37"/>
+      <c r="E39" s="37"/>
+      <c r="F39" s="37"/>
+      <c r="L39" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="M39" s="33"/>
+      <c r="N39" s="33"/>
       <c r="O39" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="P39" s="13" t="s">
+      <c r="P39" s="12" t="s">
         <v>66</v>
       </c>
       <c r="Q39" s="10" t="s">
@@ -2675,128 +2686,128 @@
       <c r="R39" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="S39" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="T39" s="14"/>
+      <c r="S39" s="36" t="s">
+        <v>63</v>
+      </c>
+      <c r="T39" s="36"/>
       <c r="U39" s="10" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="40" spans="1:21" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="27" t="s">
+      <c r="A40" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="B40" s="27"/>
-      <c r="C40" s="27"/>
-      <c r="D40" s="27"/>
-      <c r="E40" s="27"/>
-      <c r="F40" s="27"/>
-      <c r="G40" s="27"/>
-      <c r="H40" s="27"/>
-      <c r="I40" s="27"/>
-      <c r="J40" s="27"/>
+      <c r="B40" s="16"/>
+      <c r="C40" s="16"/>
+      <c r="D40" s="16"/>
+      <c r="E40" s="16"/>
+      <c r="F40" s="16"/>
+      <c r="G40" s="16"/>
+      <c r="H40" s="16"/>
+      <c r="I40" s="16"/>
+      <c r="J40" s="16"/>
       <c r="K40" s="2"/>
-      <c r="L40" s="27" t="s">
+      <c r="L40" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="M40" s="27"/>
-      <c r="N40" s="27"/>
-      <c r="O40" s="27"/>
-      <c r="P40" s="27"/>
-      <c r="Q40" s="27"/>
-      <c r="R40" s="27"/>
-      <c r="S40" s="27"/>
-      <c r="T40" s="27"/>
-      <c r="U40" s="27"/>
+      <c r="M40" s="16"/>
+      <c r="N40" s="16"/>
+      <c r="O40" s="16"/>
+      <c r="P40" s="16"/>
+      <c r="Q40" s="16"/>
+      <c r="R40" s="16"/>
+      <c r="S40" s="16"/>
+      <c r="T40" s="16"/>
+      <c r="U40" s="16"/>
     </row>
     <row r="41" spans="1:21" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="19" t="s">
+      <c r="A41" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="B41" s="19"/>
-      <c r="C41" s="19"/>
-      <c r="D41" s="26" t="s">
+      <c r="B41" s="29"/>
+      <c r="C41" s="29"/>
+      <c r="D41" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="E41" s="26"/>
-      <c r="F41" s="26"/>
-      <c r="G41" s="19" t="s">
+      <c r="E41" s="30"/>
+      <c r="F41" s="30"/>
+      <c r="G41" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="H41" s="26" t="s">
+      <c r="H41" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="I41" s="26"/>
-      <c r="J41" s="28" t="s">
+      <c r="I41" s="30"/>
+      <c r="J41" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="L41" s="26" t="s">
+      <c r="L41" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="M41" s="26"/>
-      <c r="N41" s="26"/>
-      <c r="O41" s="11" t="s">
+      <c r="M41" s="30"/>
+      <c r="N41" s="30"/>
+      <c r="O41" s="48" t="s">
         <v>39</v>
       </c>
-      <c r="P41" s="26" t="s">
+      <c r="P41" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="Q41" s="26"/>
-      <c r="R41" s="26"/>
-      <c r="S41" s="26"/>
-      <c r="T41" s="26"/>
-      <c r="U41" s="26"/>
+      <c r="Q41" s="30"/>
+      <c r="R41" s="30"/>
+      <c r="S41" s="30"/>
+      <c r="T41" s="30"/>
+      <c r="U41" s="30"/>
     </row>
     <row r="42" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="19"/>
-      <c r="B42" s="19"/>
-      <c r="C42" s="19"/>
-      <c r="D42" s="9" t="s">
+      <c r="A42" s="29"/>
+      <c r="B42" s="29"/>
+      <c r="C42" s="29"/>
+      <c r="D42" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="E42" s="19" t="s">
+      <c r="E42" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="F42" s="19"/>
-      <c r="G42" s="19"/>
-      <c r="H42" s="9" t="s">
+      <c r="F42" s="29"/>
+      <c r="G42" s="47"/>
+      <c r="H42" s="46" t="s">
         <v>33</v>
       </c>
-      <c r="I42" s="9" t="s">
+      <c r="I42" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="J42" s="28"/>
-      <c r="L42" s="14" t="s">
+      <c r="J42" s="31"/>
+      <c r="L42" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="M42" s="14"/>
-      <c r="N42" s="14"/>
+      <c r="M42" s="36"/>
+      <c r="N42" s="36"/>
       <c r="O42" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="P42" s="14" t="s">
+      <c r="P42" s="36" t="s">
         <v>67</v>
       </c>
-      <c r="Q42" s="14"/>
-      <c r="R42" s="14"/>
-      <c r="S42" s="14"/>
-      <c r="T42" s="14"/>
-      <c r="U42" s="14"/>
+      <c r="Q42" s="36"/>
+      <c r="R42" s="36"/>
+      <c r="S42" s="36"/>
+      <c r="T42" s="36"/>
+      <c r="U42" s="36"/>
     </row>
     <row r="43" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B43" s="25"/>
-      <c r="C43" s="25"/>
+      <c r="A43" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B43" s="33"/>
+      <c r="C43" s="33"/>
       <c r="D43" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E43" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F43" s="25"/>
+      <c r="E43" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F43" s="33"/>
       <c r="G43" s="10" t="s">
         <v>65</v>
       </c>
@@ -2809,34 +2820,34 @@
       <c r="J43" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L43" s="14"/>
-      <c r="M43" s="14"/>
-      <c r="N43" s="14"/>
+      <c r="L43" s="36"/>
+      <c r="M43" s="36"/>
+      <c r="N43" s="36"/>
       <c r="O43" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="P43" s="14" t="s">
+      <c r="P43" s="36" t="s">
         <v>67</v>
       </c>
-      <c r="Q43" s="14"/>
-      <c r="R43" s="14"/>
-      <c r="S43" s="14"/>
-      <c r="T43" s="14"/>
-      <c r="U43" s="14"/>
+      <c r="Q43" s="36"/>
+      <c r="R43" s="36"/>
+      <c r="S43" s="36"/>
+      <c r="T43" s="36"/>
+      <c r="U43" s="36"/>
     </row>
     <row r="44" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B44" s="25"/>
-      <c r="C44" s="25"/>
+      <c r="A44" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B44" s="33"/>
+      <c r="C44" s="33"/>
       <c r="D44" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E44" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F44" s="25"/>
+      <c r="E44" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F44" s="33"/>
       <c r="G44" s="10" t="s">
         <v>65</v>
       </c>
@@ -2849,34 +2860,34 @@
       <c r="J44" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L44" s="14"/>
-      <c r="M44" s="14"/>
-      <c r="N44" s="14"/>
+      <c r="L44" s="36"/>
+      <c r="M44" s="36"/>
+      <c r="N44" s="36"/>
       <c r="O44" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="P44" s="14" t="s">
+      <c r="P44" s="36" t="s">
         <v>67</v>
       </c>
-      <c r="Q44" s="14"/>
-      <c r="R44" s="14"/>
-      <c r="S44" s="14"/>
-      <c r="T44" s="14"/>
-      <c r="U44" s="14"/>
+      <c r="Q44" s="36"/>
+      <c r="R44" s="36"/>
+      <c r="S44" s="36"/>
+      <c r="T44" s="36"/>
+      <c r="U44" s="36"/>
     </row>
     <row r="45" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B45" s="25"/>
-      <c r="C45" s="25"/>
+      <c r="A45" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B45" s="33"/>
+      <c r="C45" s="33"/>
       <c r="D45" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E45" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F45" s="25"/>
+      <c r="E45" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F45" s="33"/>
       <c r="G45" s="10" t="s">
         <v>65</v>
       </c>
@@ -2889,34 +2900,34 @@
       <c r="J45" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L45" s="14"/>
-      <c r="M45" s="14"/>
-      <c r="N45" s="14"/>
+      <c r="L45" s="36"/>
+      <c r="M45" s="36"/>
+      <c r="N45" s="36"/>
       <c r="O45" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="P45" s="14" t="s">
+      <c r="P45" s="36" t="s">
         <v>67</v>
       </c>
-      <c r="Q45" s="14"/>
-      <c r="R45" s="14"/>
-      <c r="S45" s="14"/>
-      <c r="T45" s="14"/>
-      <c r="U45" s="14"/>
+      <c r="Q45" s="36"/>
+      <c r="R45" s="36"/>
+      <c r="S45" s="36"/>
+      <c r="T45" s="36"/>
+      <c r="U45" s="36"/>
     </row>
     <row r="46" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B46" s="25"/>
-      <c r="C46" s="25"/>
+      <c r="A46" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B46" s="33"/>
+      <c r="C46" s="33"/>
       <c r="D46" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E46" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F46" s="25"/>
+      <c r="E46" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F46" s="33"/>
       <c r="G46" s="10" t="s">
         <v>65</v>
       </c>
@@ -2929,34 +2940,34 @@
       <c r="J46" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L46" s="14"/>
-      <c r="M46" s="14"/>
-      <c r="N46" s="14"/>
+      <c r="L46" s="36"/>
+      <c r="M46" s="36"/>
+      <c r="N46" s="36"/>
       <c r="O46" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="P46" s="14" t="s">
+      <c r="P46" s="36" t="s">
         <v>67</v>
       </c>
-      <c r="Q46" s="14"/>
-      <c r="R46" s="14"/>
-      <c r="S46" s="14"/>
-      <c r="T46" s="14"/>
-      <c r="U46" s="14"/>
+      <c r="Q46" s="36"/>
+      <c r="R46" s="36"/>
+      <c r="S46" s="36"/>
+      <c r="T46" s="36"/>
+      <c r="U46" s="36"/>
     </row>
     <row r="47" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B47" s="25"/>
-      <c r="C47" s="25"/>
+      <c r="A47" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B47" s="33"/>
+      <c r="C47" s="33"/>
       <c r="D47" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E47" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F47" s="25"/>
+      <c r="E47" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F47" s="33"/>
       <c r="G47" s="10" t="s">
         <v>65</v>
       </c>
@@ -2969,38 +2980,38 @@
       <c r="J47" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L47" s="26" t="s">
+      <c r="L47" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="M47" s="26"/>
-      <c r="N47" s="26"/>
-      <c r="O47" s="11" t="s">
+      <c r="M47" s="30"/>
+      <c r="N47" s="30"/>
+      <c r="O47" s="48" t="s">
         <v>39</v>
       </c>
-      <c r="P47" s="26" t="s">
+      <c r="P47" s="30" t="s">
         <v>47</v>
       </c>
-      <c r="Q47" s="26"/>
-      <c r="R47" s="26"/>
-      <c r="S47" s="26" t="s">
+      <c r="Q47" s="30"/>
+      <c r="R47" s="30"/>
+      <c r="S47" s="49" t="s">
         <v>40</v>
       </c>
-      <c r="T47" s="26"/>
-      <c r="U47" s="26"/>
+      <c r="T47" s="49"/>
+      <c r="U47" s="49"/>
     </row>
     <row r="48" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B48" s="25"/>
-      <c r="C48" s="25"/>
+      <c r="A48" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B48" s="33"/>
+      <c r="C48" s="33"/>
       <c r="D48" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E48" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F48" s="25"/>
+      <c r="E48" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F48" s="33"/>
       <c r="G48" s="10" t="s">
         <v>65</v>
       </c>
@@ -3013,38 +3024,38 @@
       <c r="J48" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L48" s="21" t="s">
+      <c r="L48" s="38" t="s">
         <v>48</v>
       </c>
-      <c r="M48" s="21"/>
-      <c r="N48" s="21"/>
+      <c r="M48" s="38"/>
+      <c r="N48" s="38"/>
       <c r="O48" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="P48" s="15" t="s">
+      <c r="P48" s="32" t="s">
         <v>68</v>
       </c>
-      <c r="Q48" s="15"/>
-      <c r="R48" s="15"/>
-      <c r="S48" s="14" t="s">
+      <c r="Q48" s="32"/>
+      <c r="R48" s="32"/>
+      <c r="S48" s="36" t="s">
         <v>69</v>
       </c>
-      <c r="T48" s="14"/>
-      <c r="U48" s="14"/>
+      <c r="T48" s="36"/>
+      <c r="U48" s="36"/>
     </row>
     <row r="49" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B49" s="25"/>
-      <c r="C49" s="25"/>
+      <c r="A49" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B49" s="33"/>
+      <c r="C49" s="33"/>
       <c r="D49" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E49" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F49" s="25"/>
+      <c r="E49" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F49" s="33"/>
       <c r="G49" s="10" t="s">
         <v>65</v>
       </c>
@@ -3057,36 +3068,36 @@
       <c r="J49" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L49" s="21"/>
-      <c r="M49" s="21"/>
-      <c r="N49" s="21"/>
+      <c r="L49" s="38"/>
+      <c r="M49" s="38"/>
+      <c r="N49" s="38"/>
       <c r="O49" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="P49" s="15" t="s">
+      <c r="P49" s="32" t="s">
         <v>68</v>
       </c>
-      <c r="Q49" s="15"/>
-      <c r="R49" s="15"/>
-      <c r="S49" s="14" t="s">
+      <c r="Q49" s="32"/>
+      <c r="R49" s="32"/>
+      <c r="S49" s="36" t="s">
         <v>69</v>
       </c>
-      <c r="T49" s="14"/>
-      <c r="U49" s="14"/>
+      <c r="T49" s="36"/>
+      <c r="U49" s="36"/>
     </row>
     <row r="50" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B50" s="25"/>
-      <c r="C50" s="25"/>
+      <c r="A50" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B50" s="33"/>
+      <c r="C50" s="33"/>
       <c r="D50" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E50" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F50" s="25"/>
+      <c r="E50" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F50" s="33"/>
       <c r="G50" s="10" t="s">
         <v>65</v>
       </c>
@@ -3099,36 +3110,36 @@
       <c r="J50" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L50" s="21"/>
-      <c r="M50" s="21"/>
-      <c r="N50" s="21"/>
+      <c r="L50" s="38"/>
+      <c r="M50" s="38"/>
+      <c r="N50" s="38"/>
       <c r="O50" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="P50" s="15" t="s">
+      <c r="P50" s="32" t="s">
         <v>68</v>
       </c>
-      <c r="Q50" s="15"/>
-      <c r="R50" s="15"/>
-      <c r="S50" s="14" t="s">
+      <c r="Q50" s="32"/>
+      <c r="R50" s="32"/>
+      <c r="S50" s="36" t="s">
         <v>69</v>
       </c>
-      <c r="T50" s="14"/>
-      <c r="U50" s="14"/>
+      <c r="T50" s="36"/>
+      <c r="U50" s="36"/>
     </row>
     <row r="51" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B51" s="25"/>
-      <c r="C51" s="25"/>
+      <c r="A51" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B51" s="33"/>
+      <c r="C51" s="33"/>
       <c r="D51" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E51" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F51" s="25"/>
+      <c r="E51" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F51" s="33"/>
       <c r="G51" s="10" t="s">
         <v>65</v>
       </c>
@@ -3141,36 +3152,36 @@
       <c r="J51" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L51" s="21"/>
-      <c r="M51" s="21"/>
-      <c r="N51" s="21"/>
+      <c r="L51" s="38"/>
+      <c r="M51" s="38"/>
+      <c r="N51" s="38"/>
       <c r="O51" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="P51" s="15" t="s">
+      <c r="P51" s="32" t="s">
         <v>68</v>
       </c>
-      <c r="Q51" s="15"/>
-      <c r="R51" s="15"/>
-      <c r="S51" s="14" t="s">
+      <c r="Q51" s="32"/>
+      <c r="R51" s="32"/>
+      <c r="S51" s="36" t="s">
         <v>69</v>
       </c>
-      <c r="T51" s="14"/>
-      <c r="U51" s="14"/>
+      <c r="T51" s="36"/>
+      <c r="U51" s="36"/>
     </row>
     <row r="52" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B52" s="25"/>
-      <c r="C52" s="25"/>
+      <c r="A52" s="33" t="s">
+        <v>64</v>
+      </c>
+      <c r="B52" s="33"/>
+      <c r="C52" s="33"/>
       <c r="D52" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E52" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="F52" s="25"/>
+      <c r="E52" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="F52" s="33"/>
       <c r="G52" s="10" t="s">
         <v>65</v>
       </c>
@@ -3183,441 +3194,352 @@
       <c r="J52" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="L52" s="22"/>
-      <c r="M52" s="22"/>
-      <c r="N52" s="22"/>
-      <c r="O52" s="12" t="s">
+      <c r="L52" s="39"/>
+      <c r="M52" s="39"/>
+      <c r="N52" s="39"/>
+      <c r="O52" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="P52" s="15" t="s">
+      <c r="P52" s="32" t="s">
         <v>68</v>
       </c>
-      <c r="Q52" s="15"/>
-      <c r="R52" s="15"/>
-      <c r="S52" s="14" t="s">
+      <c r="Q52" s="32"/>
+      <c r="R52" s="32"/>
+      <c r="S52" s="36" t="s">
         <v>69</v>
       </c>
-      <c r="T52" s="14"/>
-      <c r="U52" s="14"/>
+      <c r="T52" s="36"/>
+      <c r="U52" s="36"/>
     </row>
     <row r="53" spans="1:21" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="16" t="s">
+      <c r="A53" s="40" t="s">
         <v>49</v>
       </c>
-      <c r="B53" s="17"/>
-      <c r="C53" s="17"/>
-      <c r="D53" s="17"/>
-      <c r="E53" s="17"/>
-      <c r="F53" s="17"/>
-      <c r="G53" s="17"/>
-      <c r="H53" s="17"/>
-      <c r="I53" s="17"/>
-      <c r="J53" s="17"/>
-      <c r="K53" s="17"/>
-      <c r="L53" s="17"/>
-      <c r="M53" s="17"/>
-      <c r="N53" s="17"/>
-      <c r="O53" s="17"/>
-      <c r="P53" s="19" t="s">
+      <c r="B53" s="41"/>
+      <c r="C53" s="41"/>
+      <c r="D53" s="41"/>
+      <c r="E53" s="41"/>
+      <c r="F53" s="41"/>
+      <c r="G53" s="41"/>
+      <c r="H53" s="41"/>
+      <c r="I53" s="41"/>
+      <c r="J53" s="41"/>
+      <c r="K53" s="41"/>
+      <c r="L53" s="41"/>
+      <c r="M53" s="41"/>
+      <c r="N53" s="41"/>
+      <c r="O53" s="41"/>
+      <c r="P53" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="Q53" s="19"/>
-      <c r="R53" s="19"/>
-      <c r="S53" s="19" t="s">
+      <c r="Q53" s="29"/>
+      <c r="R53" s="29"/>
+      <c r="S53" s="29" t="s">
         <v>70</v>
       </c>
-      <c r="T53" s="19"/>
-      <c r="U53" s="19"/>
+      <c r="T53" s="29"/>
+      <c r="U53" s="29"/>
     </row>
     <row r="54" spans="1:21" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="17"/>
-      <c r="B54" s="17"/>
-      <c r="C54" s="17"/>
-      <c r="D54" s="17"/>
-      <c r="E54" s="17"/>
-      <c r="F54" s="17"/>
-      <c r="G54" s="17"/>
-      <c r="H54" s="17"/>
-      <c r="I54" s="17"/>
-      <c r="J54" s="17"/>
-      <c r="K54" s="18"/>
-      <c r="L54" s="17"/>
-      <c r="M54" s="17"/>
-      <c r="N54" s="17"/>
-      <c r="O54" s="17"/>
-      <c r="P54" s="19"/>
-      <c r="Q54" s="19"/>
-      <c r="R54" s="19"/>
-      <c r="S54" s="19"/>
-      <c r="T54" s="19"/>
-      <c r="U54" s="19"/>
+      <c r="A54" s="41"/>
+      <c r="B54" s="41"/>
+      <c r="C54" s="41"/>
+      <c r="D54" s="41"/>
+      <c r="E54" s="41"/>
+      <c r="F54" s="41"/>
+      <c r="G54" s="41"/>
+      <c r="H54" s="41"/>
+      <c r="I54" s="41"/>
+      <c r="J54" s="41"/>
+      <c r="K54" s="42"/>
+      <c r="L54" s="41"/>
+      <c r="M54" s="41"/>
+      <c r="N54" s="41"/>
+      <c r="O54" s="41"/>
+      <c r="P54" s="29"/>
+      <c r="Q54" s="29"/>
+      <c r="R54" s="29"/>
+      <c r="S54" s="29"/>
+      <c r="T54" s="29"/>
+      <c r="U54" s="29"/>
     </row>
     <row r="55" spans="1:21" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="20" t="s">
+      <c r="A55" s="43" t="s">
         <v>51</v>
       </c>
-      <c r="B55" s="20"/>
-      <c r="C55" s="20"/>
-      <c r="D55" s="20"/>
-      <c r="E55" s="20"/>
-      <c r="F55" s="20"/>
-      <c r="G55" s="20"/>
-      <c r="H55" s="20"/>
-      <c r="I55" s="20"/>
-      <c r="J55" s="20"/>
-      <c r="L55" s="19" t="s">
+      <c r="B55" s="43"/>
+      <c r="C55" s="43"/>
+      <c r="D55" s="43"/>
+      <c r="E55" s="43"/>
+      <c r="F55" s="43"/>
+      <c r="G55" s="43"/>
+      <c r="H55" s="43"/>
+      <c r="I55" s="43"/>
+      <c r="J55" s="43"/>
+      <c r="L55" s="29" t="s">
         <v>52</v>
       </c>
-      <c r="M55" s="19"/>
-      <c r="N55" s="19"/>
-      <c r="O55" s="19"/>
-      <c r="P55" s="19"/>
-      <c r="Q55" s="19"/>
-      <c r="R55" s="19"/>
-      <c r="S55" s="19"/>
-      <c r="T55" s="19"/>
-      <c r="U55" s="19"/>
+      <c r="M55" s="29"/>
+      <c r="N55" s="29"/>
+      <c r="O55" s="29"/>
+      <c r="P55" s="29"/>
+      <c r="Q55" s="29"/>
+      <c r="R55" s="29"/>
+      <c r="S55" s="29"/>
+      <c r="T55" s="29"/>
+      <c r="U55" s="29"/>
     </row>
     <row r="56" spans="1:21" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="14" t="s">
+      <c r="A56" s="36" t="s">
         <v>53</v>
       </c>
-      <c r="B56" s="14"/>
-      <c r="C56" s="14"/>
-      <c r="D56" s="14"/>
-      <c r="E56" s="21" t="s">
+      <c r="B56" s="36"/>
+      <c r="C56" s="36"/>
+      <c r="D56" s="36"/>
+      <c r="E56" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="F56" s="21"/>
-      <c r="G56" s="21"/>
-      <c r="H56" s="21"/>
-      <c r="I56" s="21"/>
-      <c r="J56" s="21"/>
-      <c r="L56" s="14" t="s">
+      <c r="F56" s="38"/>
+      <c r="G56" s="38"/>
+      <c r="H56" s="38"/>
+      <c r="I56" s="38"/>
+      <c r="J56" s="38"/>
+      <c r="L56" s="36" t="s">
         <v>53</v>
       </c>
-      <c r="M56" s="14"/>
-      <c r="N56" s="14"/>
-      <c r="O56" s="14"/>
-      <c r="P56" s="21" t="s">
+      <c r="M56" s="36"/>
+      <c r="N56" s="36"/>
+      <c r="O56" s="36"/>
+      <c r="P56" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="Q56" s="21"/>
-      <c r="R56" s="21"/>
-      <c r="S56" s="21"/>
-      <c r="T56" s="21"/>
-      <c r="U56" s="21"/>
+      <c r="Q56" s="38"/>
+      <c r="R56" s="38"/>
+      <c r="S56" s="38"/>
+      <c r="T56" s="38"/>
+      <c r="U56" s="38"/>
     </row>
     <row r="57" spans="1:21" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="23" t="s">
+      <c r="A57" s="44" t="s">
         <v>56</v>
       </c>
-      <c r="B57" s="23"/>
-      <c r="C57" s="23"/>
-      <c r="D57" s="23"/>
-      <c r="E57" s="21"/>
-      <c r="F57" s="21"/>
-      <c r="G57" s="21"/>
-      <c r="H57" s="21"/>
-      <c r="I57" s="21"/>
-      <c r="J57" s="21"/>
-      <c r="L57" s="23" t="s">
+      <c r="B57" s="44"/>
+      <c r="C57" s="44"/>
+      <c r="D57" s="44"/>
+      <c r="E57" s="38"/>
+      <c r="F57" s="38"/>
+      <c r="G57" s="38"/>
+      <c r="H57" s="38"/>
+      <c r="I57" s="38"/>
+      <c r="J57" s="38"/>
+      <c r="L57" s="44" t="s">
         <v>56</v>
       </c>
-      <c r="M57" s="23"/>
-      <c r="N57" s="23"/>
-      <c r="O57" s="23"/>
-      <c r="P57" s="21"/>
-      <c r="Q57" s="21"/>
-      <c r="R57" s="21"/>
-      <c r="S57" s="21"/>
-      <c r="T57" s="21"/>
-      <c r="U57" s="21"/>
+      <c r="M57" s="44"/>
+      <c r="N57" s="44"/>
+      <c r="O57" s="44"/>
+      <c r="P57" s="38"/>
+      <c r="Q57" s="38"/>
+      <c r="R57" s="38"/>
+      <c r="S57" s="38"/>
+      <c r="T57" s="38"/>
+      <c r="U57" s="38"/>
     </row>
     <row r="58" spans="1:21" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="15"/>
-      <c r="B58" s="15"/>
-      <c r="C58" s="15"/>
-      <c r="D58" s="15"/>
-      <c r="E58" s="21"/>
-      <c r="F58" s="21"/>
-      <c r="G58" s="21"/>
-      <c r="H58" s="21"/>
-      <c r="I58" s="21"/>
-      <c r="J58" s="21"/>
-      <c r="L58" s="15"/>
-      <c r="M58" s="15"/>
-      <c r="N58" s="15"/>
-      <c r="O58" s="15"/>
-      <c r="P58" s="21"/>
-      <c r="Q58" s="21"/>
-      <c r="R58" s="21"/>
-      <c r="S58" s="21"/>
-      <c r="T58" s="21"/>
-      <c r="U58" s="21"/>
+      <c r="A58" s="32"/>
+      <c r="B58" s="32"/>
+      <c r="C58" s="32"/>
+      <c r="D58" s="32"/>
+      <c r="E58" s="38"/>
+      <c r="F58" s="38"/>
+      <c r="G58" s="38"/>
+      <c r="H58" s="38"/>
+      <c r="I58" s="38"/>
+      <c r="J58" s="38"/>
+      <c r="L58" s="32"/>
+      <c r="M58" s="32"/>
+      <c r="N58" s="32"/>
+      <c r="O58" s="32"/>
+      <c r="P58" s="38"/>
+      <c r="Q58" s="38"/>
+      <c r="R58" s="38"/>
+      <c r="S58" s="38"/>
+      <c r="T58" s="38"/>
+      <c r="U58" s="38"/>
     </row>
     <row r="59" spans="1:21" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="23" t="s">
+      <c r="A59" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="B59" s="23"/>
-      <c r="C59" s="23"/>
-      <c r="D59" s="23"/>
-      <c r="E59" s="21"/>
-      <c r="F59" s="21"/>
-      <c r="G59" s="21"/>
-      <c r="H59" s="21"/>
-      <c r="I59" s="21"/>
-      <c r="J59" s="21"/>
-      <c r="L59" s="23" t="s">
+      <c r="B59" s="44"/>
+      <c r="C59" s="44"/>
+      <c r="D59" s="44"/>
+      <c r="E59" s="38"/>
+      <c r="F59" s="38"/>
+      <c r="G59" s="38"/>
+      <c r="H59" s="38"/>
+      <c r="I59" s="38"/>
+      <c r="J59" s="38"/>
+      <c r="L59" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="M59" s="23"/>
-      <c r="N59" s="23"/>
-      <c r="O59" s="23"/>
-      <c r="P59" s="21"/>
-      <c r="Q59" s="21"/>
-      <c r="R59" s="21"/>
-      <c r="S59" s="21"/>
-      <c r="T59" s="21"/>
-      <c r="U59" s="21"/>
+      <c r="M59" s="44"/>
+      <c r="N59" s="44"/>
+      <c r="O59" s="44"/>
+      <c r="P59" s="38"/>
+      <c r="Q59" s="38"/>
+      <c r="R59" s="38"/>
+      <c r="S59" s="38"/>
+      <c r="T59" s="38"/>
+      <c r="U59" s="38"/>
     </row>
     <row r="60" spans="1:21" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="23"/>
-      <c r="B60" s="23"/>
-      <c r="C60" s="23"/>
-      <c r="D60" s="23"/>
-      <c r="E60" s="21"/>
-      <c r="F60" s="21"/>
-      <c r="G60" s="21"/>
-      <c r="H60" s="21"/>
-      <c r="I60" s="21"/>
-      <c r="J60" s="21"/>
-      <c r="L60" s="23"/>
-      <c r="M60" s="23"/>
-      <c r="N60" s="23"/>
-      <c r="O60" s="23"/>
-      <c r="P60" s="21"/>
-      <c r="Q60" s="21"/>
-      <c r="R60" s="21"/>
-      <c r="S60" s="21"/>
-      <c r="T60" s="21"/>
-      <c r="U60" s="21"/>
+      <c r="A60" s="44"/>
+      <c r="B60" s="44"/>
+      <c r="C60" s="44"/>
+      <c r="D60" s="44"/>
+      <c r="E60" s="38"/>
+      <c r="F60" s="38"/>
+      <c r="G60" s="38"/>
+      <c r="H60" s="38"/>
+      <c r="I60" s="38"/>
+      <c r="J60" s="38"/>
+      <c r="L60" s="44"/>
+      <c r="M60" s="44"/>
+      <c r="N60" s="44"/>
+      <c r="O60" s="44"/>
+      <c r="P60" s="38"/>
+      <c r="Q60" s="38"/>
+      <c r="R60" s="38"/>
+      <c r="S60" s="38"/>
+      <c r="T60" s="38"/>
+      <c r="U60" s="38"/>
     </row>
     <row r="61" spans="1:21" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="23" t="s">
+      <c r="A61" s="44" t="s">
         <v>57</v>
       </c>
-      <c r="B61" s="23"/>
-      <c r="C61" s="23"/>
-      <c r="D61" s="23"/>
-      <c r="E61" s="21"/>
-      <c r="F61" s="21"/>
-      <c r="G61" s="21"/>
-      <c r="H61" s="21"/>
-      <c r="I61" s="21"/>
-      <c r="J61" s="21"/>
-      <c r="L61" s="23" t="s">
+      <c r="B61" s="44"/>
+      <c r="C61" s="44"/>
+      <c r="D61" s="44"/>
+      <c r="E61" s="38"/>
+      <c r="F61" s="38"/>
+      <c r="G61" s="38"/>
+      <c r="H61" s="38"/>
+      <c r="I61" s="38"/>
+      <c r="J61" s="38"/>
+      <c r="L61" s="44" t="s">
         <v>57</v>
       </c>
-      <c r="M61" s="23"/>
-      <c r="N61" s="23"/>
-      <c r="O61" s="23"/>
-      <c r="P61" s="21"/>
-      <c r="Q61" s="21"/>
-      <c r="R61" s="21"/>
-      <c r="S61" s="21"/>
-      <c r="T61" s="21"/>
-      <c r="U61" s="21"/>
+      <c r="M61" s="44"/>
+      <c r="N61" s="44"/>
+      <c r="O61" s="44"/>
+      <c r="P61" s="38"/>
+      <c r="Q61" s="38"/>
+      <c r="R61" s="38"/>
+      <c r="S61" s="38"/>
+      <c r="T61" s="38"/>
+      <c r="U61" s="38"/>
     </row>
     <row r="62" spans="1:21" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="24" t="s">
+      <c r="A62" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="B62" s="24"/>
-      <c r="C62" s="24"/>
-      <c r="D62" s="24"/>
-      <c r="E62" s="22"/>
-      <c r="F62" s="22"/>
-      <c r="G62" s="22"/>
-      <c r="H62" s="22"/>
-      <c r="I62" s="22"/>
-      <c r="J62" s="22"/>
-      <c r="L62" s="24" t="s">
+      <c r="B62" s="45"/>
+      <c r="C62" s="45"/>
+      <c r="D62" s="45"/>
+      <c r="E62" s="39"/>
+      <c r="F62" s="39"/>
+      <c r="G62" s="39"/>
+      <c r="H62" s="39"/>
+      <c r="I62" s="39"/>
+      <c r="J62" s="39"/>
+      <c r="L62" s="45" t="s">
         <v>58</v>
       </c>
-      <c r="M62" s="24"/>
-      <c r="N62" s="24"/>
-      <c r="O62" s="24"/>
-      <c r="P62" s="22"/>
-      <c r="Q62" s="22"/>
-      <c r="R62" s="22"/>
-      <c r="S62" s="22"/>
-      <c r="T62" s="22"/>
-      <c r="U62" s="22"/>
+      <c r="M62" s="45"/>
+      <c r="N62" s="45"/>
+      <c r="O62" s="45"/>
+      <c r="P62" s="39"/>
+      <c r="Q62" s="39"/>
+      <c r="R62" s="39"/>
+      <c r="S62" s="39"/>
+      <c r="T62" s="39"/>
+      <c r="U62" s="39"/>
     </row>
     <row r="63" spans="1:21" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="14"/>
-      <c r="B63" s="14"/>
-      <c r="C63" s="14"/>
-      <c r="D63" s="14"/>
-      <c r="E63" s="14"/>
-      <c r="F63" s="14"/>
-      <c r="G63" s="14"/>
-      <c r="H63" s="14"/>
-      <c r="I63" s="14"/>
-      <c r="J63" s="14"/>
-      <c r="K63" s="14"/>
-      <c r="L63" s="14"/>
-      <c r="M63" s="14"/>
-      <c r="N63" s="14"/>
-      <c r="O63" s="14"/>
-      <c r="P63" s="14"/>
-      <c r="Q63" s="14"/>
-      <c r="R63" s="14"/>
-      <c r="S63" s="14"/>
-      <c r="T63" s="14"/>
-      <c r="U63" s="14"/>
+      <c r="A63" s="36"/>
+      <c r="B63" s="36"/>
+      <c r="C63" s="36"/>
+      <c r="D63" s="36"/>
+      <c r="E63" s="36"/>
+      <c r="F63" s="36"/>
+      <c r="G63" s="36"/>
+      <c r="H63" s="36"/>
+      <c r="I63" s="36"/>
+      <c r="J63" s="36"/>
+      <c r="K63" s="36"/>
+      <c r="L63" s="36"/>
+      <c r="M63" s="36"/>
+      <c r="N63" s="36"/>
+      <c r="O63" s="36"/>
+      <c r="P63" s="36"/>
+      <c r="Q63" s="36"/>
+      <c r="R63" s="36"/>
+      <c r="S63" s="36"/>
+      <c r="T63" s="36"/>
+      <c r="U63" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="209">
-    <mergeCell ref="J1:U1"/>
-    <mergeCell ref="K2:M2"/>
-    <mergeCell ref="N2:Q2"/>
-    <mergeCell ref="R2:S2"/>
-    <mergeCell ref="T2:U2"/>
-    <mergeCell ref="J3:M3"/>
-    <mergeCell ref="N3:U3"/>
-    <mergeCell ref="A5:U5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="I6:U6"/>
-    <mergeCell ref="C7:N7"/>
-    <mergeCell ref="O7:P7"/>
-    <mergeCell ref="Q7:U7"/>
-    <mergeCell ref="C8:H8"/>
-    <mergeCell ref="M8:N8"/>
-    <mergeCell ref="O8:P8"/>
-    <mergeCell ref="Q8:U8"/>
-    <mergeCell ref="A9:U9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="H10:L10"/>
-    <mergeCell ref="M10:U10"/>
-    <mergeCell ref="B11:J11"/>
-    <mergeCell ref="M11:U11"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="J12:M12"/>
-    <mergeCell ref="O12:U12"/>
-    <mergeCell ref="A13:J13"/>
-    <mergeCell ref="M13:P13"/>
-    <mergeCell ref="Q13:T13"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="M14:P14"/>
-    <mergeCell ref="Q14:T14"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="G15:I15"/>
-    <mergeCell ref="M15:P15"/>
-    <mergeCell ref="Q15:T15"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="M16:P16"/>
-    <mergeCell ref="Q16:T16"/>
-    <mergeCell ref="A17:U17"/>
-    <mergeCell ref="A18:J18"/>
-    <mergeCell ref="L18:U18"/>
-    <mergeCell ref="A19:C20"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="L19:N20"/>
-    <mergeCell ref="O19:P19"/>
-    <mergeCell ref="R19:T19"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="Q19:Q20"/>
-    <mergeCell ref="S20:T20"/>
-    <mergeCell ref="U19:U20"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="L21:N21"/>
-    <mergeCell ref="S21:T21"/>
-    <mergeCell ref="A22:C22"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="L22:N22"/>
-    <mergeCell ref="S22:T22"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="L23:N23"/>
-    <mergeCell ref="S23:T23"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="L24:N24"/>
-    <mergeCell ref="S24:T24"/>
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="L25:N25"/>
-    <mergeCell ref="S25:T25"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="L26:N26"/>
-    <mergeCell ref="S26:T26"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="L27:N27"/>
-    <mergeCell ref="S27:T27"/>
-    <mergeCell ref="A28:J28"/>
-    <mergeCell ref="L28:U28"/>
-    <mergeCell ref="A29:C30"/>
-    <mergeCell ref="D29:F29"/>
-    <mergeCell ref="H29:I29"/>
-    <mergeCell ref="L29:N30"/>
-    <mergeCell ref="O29:P29"/>
-    <mergeCell ref="R29:T29"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="G29:G30"/>
-    <mergeCell ref="J29:J30"/>
-    <mergeCell ref="Q29:Q30"/>
-    <mergeCell ref="S30:T30"/>
-    <mergeCell ref="U29:U30"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="L31:N31"/>
-    <mergeCell ref="S31:T31"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="E32:F32"/>
-    <mergeCell ref="L32:N32"/>
-    <mergeCell ref="S32:T32"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="L33:N33"/>
-    <mergeCell ref="S33:T33"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="L34:N34"/>
-    <mergeCell ref="S34:T34"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="L35:N35"/>
-    <mergeCell ref="S35:T35"/>
-    <mergeCell ref="A36:C36"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="L36:N36"/>
-    <mergeCell ref="S36:T36"/>
-    <mergeCell ref="A37:C37"/>
-    <mergeCell ref="E37:F37"/>
-    <mergeCell ref="L37:N37"/>
-    <mergeCell ref="S37:T37"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="E38:F38"/>
-    <mergeCell ref="L38:N38"/>
-    <mergeCell ref="S38:T38"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="L39:N39"/>
-    <mergeCell ref="S39:T39"/>
+    <mergeCell ref="A63:U63"/>
+    <mergeCell ref="P52:R52"/>
+    <mergeCell ref="S52:U52"/>
+    <mergeCell ref="A53:O54"/>
+    <mergeCell ref="P53:R54"/>
+    <mergeCell ref="S53:U54"/>
+    <mergeCell ref="A55:J55"/>
+    <mergeCell ref="L55:U55"/>
+    <mergeCell ref="A56:D56"/>
+    <mergeCell ref="E56:J62"/>
+    <mergeCell ref="L56:O56"/>
+    <mergeCell ref="P56:U62"/>
+    <mergeCell ref="A57:D57"/>
+    <mergeCell ref="L57:O57"/>
+    <mergeCell ref="A58:D58"/>
+    <mergeCell ref="L58:O58"/>
+    <mergeCell ref="A59:D59"/>
+    <mergeCell ref="L59:O59"/>
+    <mergeCell ref="A60:D60"/>
+    <mergeCell ref="L60:O60"/>
+    <mergeCell ref="A61:D61"/>
+    <mergeCell ref="L61:O61"/>
+    <mergeCell ref="A62:D62"/>
+    <mergeCell ref="L62:O62"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="E47:F47"/>
+    <mergeCell ref="L47:N47"/>
+    <mergeCell ref="P47:R47"/>
+    <mergeCell ref="S47:U47"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="E48:F48"/>
+    <mergeCell ref="L48:N52"/>
+    <mergeCell ref="P48:R48"/>
+    <mergeCell ref="S48:U48"/>
+    <mergeCell ref="A49:C49"/>
+    <mergeCell ref="E49:F49"/>
+    <mergeCell ref="P49:R49"/>
+    <mergeCell ref="S49:U49"/>
+    <mergeCell ref="A50:C50"/>
+    <mergeCell ref="E50:F50"/>
+    <mergeCell ref="P50:R50"/>
+    <mergeCell ref="S50:U50"/>
+    <mergeCell ref="A51:C51"/>
+    <mergeCell ref="E51:F51"/>
+    <mergeCell ref="P51:R51"/>
+    <mergeCell ref="S51:U51"/>
+    <mergeCell ref="A52:C52"/>
+    <mergeCell ref="E52:F52"/>
     <mergeCell ref="A40:J40"/>
     <mergeCell ref="L40:U40"/>
     <mergeCell ref="A41:C42"/>
@@ -3642,54 +3564,143 @@
     <mergeCell ref="A46:C46"/>
     <mergeCell ref="E46:F46"/>
     <mergeCell ref="P46:U46"/>
-    <mergeCell ref="A47:C47"/>
-    <mergeCell ref="E47:F47"/>
-    <mergeCell ref="L47:N47"/>
-    <mergeCell ref="P47:R47"/>
-    <mergeCell ref="S47:U47"/>
-    <mergeCell ref="A48:C48"/>
-    <mergeCell ref="E48:F48"/>
-    <mergeCell ref="L48:N52"/>
-    <mergeCell ref="P48:R48"/>
-    <mergeCell ref="S48:U48"/>
-    <mergeCell ref="A49:C49"/>
-    <mergeCell ref="E49:F49"/>
-    <mergeCell ref="P49:R49"/>
-    <mergeCell ref="S49:U49"/>
-    <mergeCell ref="A50:C50"/>
-    <mergeCell ref="E50:F50"/>
-    <mergeCell ref="P50:R50"/>
-    <mergeCell ref="S50:U50"/>
-    <mergeCell ref="A51:C51"/>
-    <mergeCell ref="E51:F51"/>
-    <mergeCell ref="P51:R51"/>
-    <mergeCell ref="S51:U51"/>
-    <mergeCell ref="A52:C52"/>
-    <mergeCell ref="E52:F52"/>
-    <mergeCell ref="A63:U63"/>
-    <mergeCell ref="P52:R52"/>
-    <mergeCell ref="S52:U52"/>
-    <mergeCell ref="A53:O54"/>
-    <mergeCell ref="P53:R54"/>
-    <mergeCell ref="S53:U54"/>
-    <mergeCell ref="A55:J55"/>
-    <mergeCell ref="L55:U55"/>
-    <mergeCell ref="A56:D56"/>
-    <mergeCell ref="E56:J62"/>
-    <mergeCell ref="L56:O56"/>
-    <mergeCell ref="P56:U62"/>
-    <mergeCell ref="A57:D57"/>
-    <mergeCell ref="L57:O57"/>
-    <mergeCell ref="A58:D58"/>
-    <mergeCell ref="L58:O58"/>
-    <mergeCell ref="A59:D59"/>
-    <mergeCell ref="L59:O59"/>
-    <mergeCell ref="A60:D60"/>
-    <mergeCell ref="L60:O60"/>
-    <mergeCell ref="A61:D61"/>
-    <mergeCell ref="L61:O61"/>
-    <mergeCell ref="A62:D62"/>
-    <mergeCell ref="L62:O62"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="L37:N37"/>
+    <mergeCell ref="S37:T37"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="L38:N38"/>
+    <mergeCell ref="S38:T38"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="L39:N39"/>
+    <mergeCell ref="S39:T39"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="L34:N34"/>
+    <mergeCell ref="S34:T34"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="L35:N35"/>
+    <mergeCell ref="S35:T35"/>
+    <mergeCell ref="A36:C36"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="L36:N36"/>
+    <mergeCell ref="S36:T36"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="L31:N31"/>
+    <mergeCell ref="S31:T31"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="L32:N32"/>
+    <mergeCell ref="S32:T32"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="L33:N33"/>
+    <mergeCell ref="S33:T33"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="L27:N27"/>
+    <mergeCell ref="S27:T27"/>
+    <mergeCell ref="A28:J28"/>
+    <mergeCell ref="L28:U28"/>
+    <mergeCell ref="A29:C30"/>
+    <mergeCell ref="D29:F29"/>
+    <mergeCell ref="H29:I29"/>
+    <mergeCell ref="L29:N30"/>
+    <mergeCell ref="O29:P29"/>
+    <mergeCell ref="R29:T29"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="G29:G30"/>
+    <mergeCell ref="J29:J30"/>
+    <mergeCell ref="Q29:Q30"/>
+    <mergeCell ref="S30:T30"/>
+    <mergeCell ref="U29:U30"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="L24:N24"/>
+    <mergeCell ref="S24:T24"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="L25:N25"/>
+    <mergeCell ref="S25:T25"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="L26:N26"/>
+    <mergeCell ref="S26:T26"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="L21:N21"/>
+    <mergeCell ref="S21:T21"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="L22:N22"/>
+    <mergeCell ref="S22:T22"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="L23:N23"/>
+    <mergeCell ref="S23:T23"/>
+    <mergeCell ref="A17:U17"/>
+    <mergeCell ref="A18:J18"/>
+    <mergeCell ref="L18:U18"/>
+    <mergeCell ref="A19:C20"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="L19:N20"/>
+    <mergeCell ref="O19:P19"/>
+    <mergeCell ref="R19:T19"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="Q19:Q20"/>
+    <mergeCell ref="S20:T20"/>
+    <mergeCell ref="U19:U20"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="M14:P14"/>
+    <mergeCell ref="Q14:T14"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="G15:I15"/>
+    <mergeCell ref="M15:P15"/>
+    <mergeCell ref="Q15:T15"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="M16:P16"/>
+    <mergeCell ref="Q16:T16"/>
+    <mergeCell ref="B11:J11"/>
+    <mergeCell ref="M11:U11"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="J12:M12"/>
+    <mergeCell ref="O12:U12"/>
+    <mergeCell ref="A13:J13"/>
+    <mergeCell ref="M13:P13"/>
+    <mergeCell ref="Q13:T13"/>
+    <mergeCell ref="C7:N7"/>
+    <mergeCell ref="O7:P7"/>
+    <mergeCell ref="Q7:U7"/>
+    <mergeCell ref="C8:H8"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="O8:P8"/>
+    <mergeCell ref="Q8:U8"/>
+    <mergeCell ref="A9:U9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="H10:L10"/>
+    <mergeCell ref="M10:U10"/>
+    <mergeCell ref="J1:U1"/>
+    <mergeCell ref="K2:M2"/>
+    <mergeCell ref="N2:Q2"/>
+    <mergeCell ref="R2:S2"/>
+    <mergeCell ref="T2:U2"/>
+    <mergeCell ref="J3:M3"/>
+    <mergeCell ref="N3:U3"/>
+    <mergeCell ref="A5:U5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="D6:H6"/>
+    <mergeCell ref="I6:U6"/>
   </mergeCells>
   <pageMargins left="0.2" right="0.15" top="0.2" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="14" scale="98" fitToHeight="0" orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>

</xml_diff>